<commit_message>
feat: implement achievement KPI
</commit_message>
<xml_diff>
--- a/src/Sales-Dashboard.xlsx
+++ b/src/Sales-Dashboard.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seikoatsuumi/Desktop/20260713_GitHub/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seikoatsuumi/Documents/GitHub/Sales-Dashboard/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34751C3A-5CAC-AC43-BBA2-F3051C7C492E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41306D1B-7B72-804D-BA2D-F28317562FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5020" yWindow="1800" windowWidth="28300" windowHeight="17360" xr2:uid="{DEEBA340-9C08-5045-B722-94D475730B04}"/>
+    <workbookView xWindow="8060" yWindow="2820" windowWidth="28300" windowHeight="17360" xr2:uid="{DEEBA340-9C08-5045-B722-94D475730B04}"/>
   </bookViews>
   <sheets>
     <sheet name="Home Dashboard" sheetId="3" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <definedName name="SalesReps">tblSalesReps[Sales Representatives]</definedName>
     <definedName name="SalesStatus">tblSalesStatus[Sales Status]</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -511,7 +511,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -545,19 +545,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -572,12 +560,33 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="24" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -590,40 +599,49 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="24" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="9" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1163,131 +1181,134 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1"/>
     <row r="2" spans="1:12" ht="28" customHeight="1">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
     </row>
     <row r="3" spans="1:12" ht="28" customHeight="1">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
+      <c r="A3" s="36"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
     </row>
     <row r="4" spans="1:12" ht="22" customHeight="1"/>
     <row r="5" spans="1:12" ht="20" customHeight="1">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="22" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="22" t="s">
+      <c r="E5" s="26"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="H5" s="23"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="22" t="s">
+      <c r="H5" s="26"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="K5" s="23"/>
-      <c r="L5" s="24"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" spans="1:12" ht="24" customHeight="1">
-      <c r="A6" s="19"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="21"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="17"/>
     </row>
     <row r="7" spans="1:12" ht="24" customHeight="1">
-      <c r="A7" s="26">
+      <c r="A7" s="18">
+        <f>SUM(tblSales[Revenue])</f>
         <v>0</v>
       </c>
-      <c r="B7" s="27"/>
-      <c r="C7" s="28"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="20"/>
       <c r="D7" s="29">
+        <f>SUM(tblSales[Sales])</f>
         <v>0</v>
       </c>
-      <c r="E7" s="27"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="30">
+      <c r="E7" s="19"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="34">
+        <f>SUM(tblSales[Revenue])/INDEX(tblSettings[Value],MATCH("Monthly Revenue Target",tblSettings[Setting],0))</f>
         <v>0</v>
       </c>
-      <c r="H7" s="27"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="30">
+      <c r="H7" s="39"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="34">
         <v>0</v>
       </c>
-      <c r="K7" s="27"/>
-      <c r="L7" s="28"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="20"/>
     </row>
     <row r="8" spans="1:12" ht="24" customHeight="1">
-      <c r="A8" s="31"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="27"/>
-      <c r="L8" s="28"/>
+      <c r="A8" s="21"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="20"/>
     </row>
     <row r="9" spans="1:12" ht="24" customHeight="1">
-      <c r="A9" s="32"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="37"/>
+      <c r="A9" s="22"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="32"/>
+      <c r="L9" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="22" customHeight="1">
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="10"/>
@@ -1296,12 +1317,12 @@
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="10"/>
@@ -1310,12 +1331,12 @@
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="10"/>
@@ -1324,12 +1345,12 @@
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="13"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="10"/>
@@ -1338,12 +1359,12 @@
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="10"/>
@@ -1352,12 +1373,12 @@
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="10"/>
@@ -1366,12 +1387,12 @@
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="10"/>
@@ -1380,12 +1401,12 @@
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="10"/>
@@ -1394,12 +1415,12 @@
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="13"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="10"/>
@@ -1408,12 +1429,12 @@
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11"/>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="10"/>
@@ -1422,12 +1443,12 @@
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="10"/>
@@ -1436,30 +1457,30 @@
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
     </row>
     <row r="24" spans="1:12">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="13" t="s">
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
@@ -1474,11 +1495,11 @@
       <c r="G25" t="s">
         <v>54</v>
       </c>
-      <c r="H25" s="13" t="s">
+      <c r="H25" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="I25" s="13"/>
-      <c r="J25" s="13"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11"/>
       <c r="K25" t="s">
         <v>56</v>
       </c>
@@ -1488,8 +1509,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="J5:L6"/>
-    <mergeCell ref="J7:L9"/>
     <mergeCell ref="A2:L3"/>
     <mergeCell ref="G11:L22"/>
     <mergeCell ref="A24:F24"/>
@@ -1501,6 +1520,8 @@
     <mergeCell ref="D7:F9"/>
     <mergeCell ref="G5:I6"/>
     <mergeCell ref="G7:I9"/>
+    <mergeCell ref="J5:L6"/>
+    <mergeCell ref="J7:L9"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1659,6 +1680,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
feat: implement conversion rate KPI
</commit_message>
<xml_diff>
--- a/src/Sales-Dashboard.xlsx
+++ b/src/Sales-Dashboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seikoatsuumi/Documents/GitHub/Sales-Dashboard/src/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seikoatsuumi/Documents/GitHub/00_Sales-Dashboard/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41306D1B-7B72-804D-BA2D-F28317562FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA7EE52-10CB-304F-AB4A-39974923D584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8060" yWindow="2820" windowWidth="28300" windowHeight="17360" xr2:uid="{DEEBA340-9C08-5045-B722-94D475730B04}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="61">
   <si>
     <t>Sales Representatives</t>
     <phoneticPr fontId="1"/>
@@ -545,7 +545,19 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -615,18 +627,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1181,134 +1181,135 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1"/>
     <row r="2" spans="1:12" ht="28" customHeight="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
     </row>
     <row r="3" spans="1:12" ht="28" customHeight="1">
-      <c r="A3" s="36"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
     </row>
     <row r="4" spans="1:12" ht="22" customHeight="1"/>
     <row r="5" spans="1:12" ht="20" customHeight="1">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="25" t="s">
+      <c r="B5" s="17"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="26"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="25" t="s">
+      <c r="E5" s="30"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="H5" s="26"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="25" t="s">
+      <c r="H5" s="30"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="K5" s="26"/>
-      <c r="L5" s="27"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="31"/>
     </row>
     <row r="6" spans="1:12" ht="24" customHeight="1">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="28"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="17"/>
+      <c r="A6" s="19"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="21"/>
     </row>
     <row r="7" spans="1:12" ht="24" customHeight="1">
-      <c r="A7" s="18">
+      <c r="A7" s="22">
         <f>SUM(tblSales[Revenue])</f>
         <v>0</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="29">
+      <c r="B7" s="23"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="33">
         <f>SUM(tblSales[Sales])</f>
         <v>0</v>
       </c>
-      <c r="E7" s="19"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="34">
+      <c r="E7" s="23"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="38">
         <f>SUM(tblSales[Revenue])/INDEX(tblSettings[Value],MATCH("Monthly Revenue Target",tblSettings[Setting],0))</f>
         <v>0</v>
       </c>
       <c r="H7" s="39"/>
       <c r="I7" s="40"/>
-      <c r="J7" s="34">
-        <v>0</v>
-      </c>
-      <c r="K7" s="19"/>
-      <c r="L7" s="20"/>
+      <c r="J7" s="38">
+        <f>IF(COUNTIF(tblSales[Status],"Meeting")+COUNTIF(tblSales[Status],"Won")=0,0,COUNTIF(tblSales[Status],"Won")/(COUNTIF(tblSales[Status],"Meeting")+COUNTIF(tblSales[Status],"Won")))</f>
+        <v>0.5</v>
+      </c>
+      <c r="K7" s="39"/>
+      <c r="L7" s="40"/>
     </row>
     <row r="8" spans="1:12" ht="24" customHeight="1">
-      <c r="A8" s="21"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="34"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="38"/>
       <c r="H8" s="39"/>
       <c r="I8" s="40"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="20"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="40"/>
     </row>
     <row r="9" spans="1:12" ht="24" customHeight="1">
-      <c r="A9" s="22"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="33"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="37"/>
       <c r="G9" s="41"/>
       <c r="H9" s="42"/>
       <c r="I9" s="43"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="32"/>
-      <c r="L9" s="33"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="42"/>
+      <c r="L9" s="43"/>
     </row>
     <row r="11" spans="1:12" ht="22" customHeight="1">
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="10"/>
@@ -1317,12 +1318,12 @@
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="10"/>
@@ -1331,12 +1332,12 @@
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="10"/>
@@ -1345,12 +1346,12 @@
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="10"/>
@@ -1359,12 +1360,12 @@
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="10"/>
@@ -1373,12 +1374,12 @@
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="13"/>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="10"/>
@@ -1387,12 +1388,12 @@
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="10"/>
@@ -1401,12 +1402,12 @@
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="10"/>
@@ -1415,12 +1416,12 @@
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="10"/>
@@ -1429,12 +1430,12 @@
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="10"/>
@@ -1443,12 +1444,12 @@
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="10"/>
@@ -1457,30 +1458,30 @@
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
     </row>
     <row r="24" spans="1:12">
-      <c r="A24" s="37" t="s">
+      <c r="A24" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="11" t="s">
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
@@ -1495,11 +1496,11 @@
       <c r="G25" t="s">
         <v>54</v>
       </c>
-      <c r="H25" s="11" t="s">
+      <c r="H25" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
       <c r="K25" t="s">
         <v>56</v>
       </c>
@@ -1629,15 +1630,24 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3"/>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4"/>
       <c r="B4" t="s">
         <v>57</v>
       </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5"/>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6"/>

</xml_diff>

<commit_message>
feat: finalize sales dashboard portfolio
feat: finalize sales dashboard portfolio

- finalize KPI calculations and dashboard layout
- add sales representative and weekly revenue analysis
- add dynamic recent activities
- add portfolio sample workbook
- add dashboard screenshot and architecture diagram
- update README documentation
</commit_message>
<xml_diff>
--- a/src/Sales-Dashboard.xlsx
+++ b/src/Sales-Dashboard.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seikoatsuumi/Documents/GitHub/Sales-Dashboard/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17009251-9857-EB4E-910F-58361519E0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C17DD570-B99A-CC41-BE04-AC9ACCE49249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8060" yWindow="1700" windowWidth="28300" windowHeight="18480" xr2:uid="{DEEBA340-9C08-5045-B722-94D475730B04}"/>
   </bookViews>
@@ -21,10 +21,6 @@
     <sheet name="Settings" sheetId="1" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v2.0" hidden="1">Summary!$G$1</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Summary!$G$2:$G$5</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Summary!$H$1</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Summary!$H$2:$H$5</definedName>
     <definedName name="Products">tblProducts[Product / Service]</definedName>
     <definedName name="SalesReps">tblSalesReps[Sales Representatives]</definedName>
     <definedName name="SalesStatus">tblSalesStatus[Sales Status]</definedName>
@@ -53,7 +49,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -75,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="69">
   <si>
     <t>Sales Representatives</t>
     <phoneticPr fontId="1"/>
@@ -225,14 +221,6 @@
   </si>
   <si>
     <t>Sales Dashboard</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Revenue by Week</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Top Sales Representatives</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -289,6 +277,33 @@
   </si>
   <si>
     <t>Week</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ABC Corporation</t>
+  </si>
+  <si>
+    <t>ABC Corporation</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Bright Solutions</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Northwind Ltd</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Green Field Inc</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Sunrise Trading</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Blue Ocean Partners</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -296,12 +311,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="24" formatCode="\$#,##0_);[Red]\(\$#,##0\)"/>
     <numFmt numFmtId="176" formatCode="\$#,##0.00;\-\$#,##0.00"/>
-    <numFmt numFmtId="184" formatCode="&quot;Week &quot;0"/>
+    <numFmt numFmtId="177" formatCode="&quot;Week &quot;0"/>
+    <numFmt numFmtId="178" formatCode="\$#,##0;\-\$#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -335,14 +351,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="游ゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="12"/>
       <color theme="3" tint="9.9978637043366805E-2"/>
@@ -370,7 +378,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -386,12 +394,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -576,7 +578,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -610,11 +612,20 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -625,104 +636,89 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="24" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="24" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -738,9 +734,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -845,6 +838,9 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="3" formatCode="#,##0"/>
@@ -1078,16 +1074,16 @@
                 <c:formatCode>\$#,##0.00;\-\$#,##0.00</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>8000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6</c:v>
+                  <c:v>4000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6</c:v>
+                  <c:v>6000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6</c:v>
+                  <c:v>6000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1343,15 +1339,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Summary!$G$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Week</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
+            <c:v>Revenue</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
@@ -1365,23 +1353,32 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
-          <c:val>
+          <c:cat>
             <c:numRef>
-              <c:f>Summary!$G$2:$G$5</c:f>
+              <c:f>'Weekly Summary'!$A$2:$A$3</c:f>
               <c:numCache>
-                <c:formatCode>"Week "0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>29</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>29</c:v>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Weekly Summary'!$B$2:$B$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>12000</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>29</c:v>
+                <c:pt idx="1">
+                  <c:v>12000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1389,7 +1386,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AC24-104E-8F0B-AD5BA867EC55}"/>
+              <c16:uniqueId val="{00000004-3137-8E4A-8F4F-EA44852D2527}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1412,6 +1409,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1459,6 +1457,7 @@
         <c:axId val="370169984"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1476,7 +1475,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="&quot;Week &quot;0" sourceLinked="1"/>
+        <c:numFmt formatCode="[$$]#,##0_);[Red]\([$$]#,##0\)" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2700,15 +2699,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>254000</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>142876</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>15876</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>1079500</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>47626</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2737,16 +2736,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>952499</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>158750</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>584198</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>349249</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>222250</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1066799</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2777,8 +2776,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5775A406-8C57-2D44-8E38-06F9B76A48FE}" name="tblSales" displayName="tblSales" ref="A1:N14" totalsRowShown="0" headerRowDxfId="16">
-  <autoFilter ref="A1:N14" xr:uid="{5775A406-8C57-2D44-8E38-06F9B76A48FE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5775A406-8C57-2D44-8E38-06F9B76A48FE}" name="tblSales" displayName="tblSales" ref="A1:N13" totalsRowShown="0" headerRowDxfId="16">
+  <autoFilter ref="A1:N13" xr:uid="{5775A406-8C57-2D44-8E38-06F9B76A48FE}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{7AEBEA8D-185B-E240-9B93-D5C2046F3112}" name="Date" dataDxfId="15">
       <calculatedColumnFormula>AND($A2="",COUNTA($A2:$M2)&gt;0)</calculatedColumnFormula>
@@ -2786,9 +2785,7 @@
     <tableColumn id="2" xr3:uid="{7805F7A6-3771-7C4A-8F61-0E7A67EA1F99}" name="Sales Rep" dataDxfId="14">
       <calculatedColumnFormula>COUNTIF(tblSales[Sales Rep],"Emma Smith")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{D1628122-9A8C-B44A-A564-1B2E43946958}" name="Customer / Lead" dataDxfId="13">
-      <calculatedColumnFormula>AND($B2="",COUNTA($A2:$M2)&gt;0)</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="3" xr3:uid="{D1628122-9A8C-B44A-A564-1B2E43946958}" name="Customer / Lead" dataDxfId="13"/>
     <tableColumn id="4" xr3:uid="{034F583C-403F-164E-A74E-E1921A197D5D}" name="Product / Service"/>
     <tableColumn id="5" xr3:uid="{F8EF18BD-111D-894D-92C5-E6CCD0C4603E}" name="Status"/>
     <tableColumn id="6" xr3:uid="{D190B2EA-B05C-5144-B402-F8BA1C66B7FE}" name="Calls" dataDxfId="12"/>
@@ -2799,7 +2796,7 @@
     <tableColumn id="11" xr3:uid="{3982783A-49F4-BB4E-9158-F99038DA3F59}" name="Revenue" dataDxfId="7"/>
     <tableColumn id="12" xr3:uid="{7AEC310F-1373-F74C-AA6A-951D4229DFAE}" name="Target" dataDxfId="6"/>
     <tableColumn id="13" xr3:uid="{64061935-2ABD-9C40-8E9F-1B2E101A5623}" name="Notes"/>
-    <tableColumn id="14" xr3:uid="{A63E6501-8160-114D-8405-8A1C7D3EC61F}" name="Week" dataDxfId="1">
+    <tableColumn id="14" xr3:uid="{A63E6501-8160-114D-8405-8A1C7D3EC61F}" name="Week" dataDxfId="5">
       <calculatedColumnFormula>WEEKNUM(tblSales[[#This Row],[Date]],2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2808,7 +2805,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9A85D2D1-E493-C449-AFBB-91C6C06AB33B}" name="tblSalesReps" displayName="tblSalesReps" ref="A1:B7" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9A85D2D1-E493-C449-AFBB-91C6C06AB33B}" name="tblSalesReps" displayName="tblSalesReps" ref="A1:B7" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A1:B7" xr:uid="{9A85D2D1-E493-C449-AFBB-91C6C06AB33B}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{5BDCD5EE-5B11-4A41-8E59-47765A6F863C}" name="Sales Representatives"/>
@@ -2819,7 +2816,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{051952BA-27E7-EE41-B9D1-D365838D49C4}" name="tblSalesStatus" displayName="tblSalesStatus" ref="D1:E7" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{051952BA-27E7-EE41-B9D1-D365838D49C4}" name="tblSalesStatus" displayName="tblSalesStatus" ref="D1:E7" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="D1:E7" xr:uid="{051952BA-27E7-EE41-B9D1-D365838D49C4}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{F9D67EA4-B605-FF46-94D3-C8281EEEFD46}" name="Sales Status"/>
@@ -2830,8 +2827,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{96E43BC3-EAEF-B04D-B96D-B845E0E15A9D}" name="tblProducts" displayName="tblProducts" ref="G1:H5" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="G1:H5" xr:uid="{96E43BC3-EAEF-B04D-B96D-B845E0E15A9D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{96E43BC3-EAEF-B04D-B96D-B845E0E15A9D}" name="tblProducts" displayName="tblProducts" ref="G1:H6" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="G1:H6" xr:uid="{96E43BC3-EAEF-B04D-B96D-B845E0E15A9D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{933AF870-CA0F-E24E-84CB-0076703675A6}" name="Product / Service"/>
     <tableColumn id="2" xr3:uid="{CA07CC0E-9BB2-F94B-B288-C811CF991BAA}" name="Category"/>
@@ -2841,7 +2838,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{58683640-83A2-B243-B8A9-8A2DFD09E223}" name="tblSettings" displayName="tblSettings" ref="J1:K6" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{58683640-83A2-B243-B8A9-8A2DFD09E223}" name="tblSettings" displayName="tblSettings" ref="J1:K6" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="J1:K6" xr:uid="{58683640-83A2-B243-B8A9-8A2DFD09E223}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{43274D1A-0DE2-2C49-8C45-2604541AF87E}" name="Setting"/>
@@ -3169,100 +3166,102 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE5ED206-0E71-4D40-9B9D-730A18A08815}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
-    <col min="1" max="12" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="12" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1"/>
     <row r="2" spans="1:12" ht="28" customHeight="1">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
     </row>
     <row r="3" spans="1:12" ht="28" customHeight="1">
-      <c r="A3" s="14"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="17"/>
     </row>
     <row r="4" spans="1:12" ht="22" customHeight="1"/>
     <row r="5" spans="1:12" ht="20" customHeight="1">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="20"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="33"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="33"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="31" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" s="32"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="H5" s="32"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="K5" s="32"/>
-      <c r="L5" s="33"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="34"/>
     </row>
     <row r="6" spans="1:12" ht="24" customHeight="1">
-      <c r="A6" s="21"/>
-      <c r="B6" s="22"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="23"/>
+      <c r="A6" s="22"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="24"/>
     </row>
     <row r="7" spans="1:12" ht="24" customHeight="1">
-      <c r="A7" s="24">
+      <c r="A7" s="25">
         <f>SUM(tblSales[Revenue])</f>
-        <v>26</v>
-      </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="35">
+        <v>24000</v>
+      </c>
+      <c r="B7" s="26"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="36">
         <f>SUM(tblSales[Sales])</f>
-        <v>39</v>
-      </c>
-      <c r="E7" s="25"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="40">
+        <v>36</v>
+      </c>
+      <c r="E7" s="26"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="41">
         <f>SUM(tblSales[Revenue])/INDEX(tblSettings[Value],MATCH("Monthly Revenue Target",tblSettings[Setting],0))</f>
-        <v>5.1999999999999995E-4</v>
-      </c>
-      <c r="H7" s="41"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="40">
+        <v>0.48</v>
+      </c>
+      <c r="H7" s="42"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="41">
         <f>IF(
 COUNTIF(tblSales[Status],"Meeting")
 +COUNTIF(tblSales[Status],"Won")=0,
@@ -3274,61 +3273,63 @@
 +COUNTIF(tblSales[Status],"Won")
 )
 )</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="41"/>
-      <c r="L7" s="42"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="K7" s="42"/>
+      <c r="L7" s="43"/>
     </row>
     <row r="8" spans="1:12" ht="24" customHeight="1">
-      <c r="A8" s="27"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="41"/>
-      <c r="L8" s="42"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="42"/>
+      <c r="L8" s="43"/>
     </row>
     <row r="9" spans="1:12" ht="24" customHeight="1">
-      <c r="A9" s="28"/>
-      <c r="B9" s="29"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="43"/>
-      <c r="K9" s="44"/>
-      <c r="L9" s="45"/>
+      <c r="A9" s="29"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="40"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="46"/>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="22" customHeight="1">
-      <c r="B11" s="11" t="str">
+      <c r="A11" t="str">
         <f>INDEX(Summary!$A$2:$A$5,MATCH(MAX(Summary!$B$2:$B$5),Summary!$B$2:$B$5,0))</f>
         <v>Emma Smith</v>
       </c>
+      <c r="B11" s="11">
+        <f>MAX(Summary!$B$2:$B$5)</f>
+        <v>8000</v>
+      </c>
       <c r="C11" s="10">
         <f>MAX(Summary!$B$2:$B$5)</f>
-        <v>8</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
+        <v>8000</v>
+      </c>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="18"/>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="8"/>
@@ -3337,12 +3338,12 @@
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="15"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="8"/>
@@ -3351,12 +3352,12 @@
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="15"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="8"/>
@@ -3365,12 +3366,12 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="15"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18"/>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="8"/>
@@ -3379,12 +3380,12 @@
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="8"/>
@@ -3393,12 +3394,12 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="18"/>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="8"/>
@@ -3407,12 +3408,12 @@
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="8"/>
@@ -3421,12 +3422,12 @@
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="8"/>
@@ -3435,12 +3436,12 @@
       <c r="D19" s="8"/>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="15"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="18"/>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="8"/>
@@ -3449,12 +3450,12 @@
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="15"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="18"/>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="8"/>
@@ -3463,12 +3464,12 @@
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="15"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="18"/>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="8"/>
@@ -3477,67 +3478,184 @@
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="18"/>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
     </row>
     <row r="24" spans="1:12">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" t="s">
-        <v>50</v>
-      </c>
-      <c r="E25" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" t="s">
-        <v>53</v>
-      </c>
-      <c r="B42" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C42" s="15"/>
-      <c r="D42" s="15"/>
-      <c r="E42" t="s">
-        <v>55</v>
-      </c>
-      <c r="F42" t="s">
-        <v>51</v>
-      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="7" cm="1">
+        <f t="array" ref="A28:D32">_xlfn.TAKE(
+    _xlfn.SORTBY(
+        _xlfn.CHOOSECOLS(
+            tblSales[],
+            1,
+            3,
+            5,
+            11
+        ),
+        tblSales[Date],
+        -1
+    ),
+    5
+)</f>
+        <v>46228</v>
+      </c>
+      <c r="B28" t="str">
+        <v>ABC Corporation</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D28" s="13">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="7">
+        <v>46227</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Blue Ocean Partners</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D29" s="13">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" s="7">
+        <v>46226</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Sunrise Trading</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D30" s="13">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" s="7">
+        <v>46225</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Green Field Inc</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D31" s="13">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" s="7">
+        <v>46224</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Bright Solutions</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D32" s="13">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="7"/>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="7"/>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="7"/>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="7"/>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="7"/>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="B43" s="7"/>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="B44" s="7"/>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="B45" s="7"/>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="B46" s="7"/>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="B47" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="11">
     <mergeCell ref="A2:L3"/>
     <mergeCell ref="G11:L22"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="A7:C9"/>
     <mergeCell ref="D5:F6"/>
@@ -3557,7 +3675,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F993C496-3950-8F40-8A32-2568E65126D5}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="7" bestFit="1" customWidth="1"/>
@@ -3613,7 +3731,7 @@
         <v>45</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -3623,15 +3741,14 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2">
-        <f ca="1">AND($B4="",COUNTA($A4:$M4)&gt;0)</f>
-        <v>0</v>
+      <c r="C2" t="s">
+        <v>63</v>
       </c>
       <c r="D2" t="s">
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F2" s="6">
         <v>5</v>
@@ -3649,7 +3766,7 @@
         <v>3</v>
       </c>
       <c r="K2" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L2" s="4">
         <v>2500</v>
@@ -3664,14 +3781,13 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="7">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <f t="shared" ref="C3:C14" ca="1" si="0">AND($B3="",COUNTA($A3:$M3)&gt;0)</f>
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>65</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -3695,7 +3811,7 @@
         <v>3</v>
       </c>
       <c r="K3" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L3" s="4">
         <v>2500</v>
@@ -3710,14 +3826,13 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="7">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>66</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
@@ -3741,7 +3856,7 @@
         <v>3</v>
       </c>
       <c r="K4" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L4" s="4">
         <v>2500</v>
@@ -3756,14 +3871,13 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="7">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>67</v>
       </c>
       <c r="D5" t="s">
         <v>18</v>
@@ -3787,7 +3901,7 @@
         <v>3</v>
       </c>
       <c r="K5" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L5" s="4">
         <v>2500</v>
@@ -3802,14 +3916,13 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="7">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>68</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
@@ -3833,7 +3946,7 @@
         <v>3</v>
       </c>
       <c r="K6" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L6" s="4">
         <v>2500</v>
@@ -3848,14 +3961,13 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="7">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>63</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -3879,7 +3991,7 @@
         <v>3</v>
       </c>
       <c r="K7" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L7" s="4">
         <v>2500</v>
@@ -3894,14 +4006,13 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="7">
-        <v>46222</v>
+        <v>46224</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>64</v>
       </c>
       <c r="D8" t="s">
         <v>18</v>
@@ -3925,7 +4036,7 @@
         <v>3</v>
       </c>
       <c r="K8" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L8" s="4">
         <v>2500</v>
@@ -3935,7 +4046,7 @@
       </c>
       <c r="N8">
         <f>WEEKNUM(tblSales[[#This Row],[Date]],2)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -3943,11 +4054,10 @@
         <v>46224</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>65</v>
       </c>
       <c r="D9" t="s">
         <v>18</v>
@@ -3971,7 +4081,7 @@
         <v>3</v>
       </c>
       <c r="K9" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L9" s="4">
         <v>2500</v>
@@ -3986,14 +4096,13 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="7">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>66</v>
       </c>
       <c r="D10" t="s">
         <v>18</v>
@@ -4017,7 +4126,7 @@
         <v>3</v>
       </c>
       <c r="K10" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L10" s="4">
         <v>2500</v>
@@ -4032,14 +4141,13 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="7">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
       </c>
       <c r="D11" t="s">
         <v>18</v>
@@ -4063,7 +4171,7 @@
         <v>3</v>
       </c>
       <c r="K11" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L11" s="4">
         <v>2500</v>
@@ -4078,14 +4186,13 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="7">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
       </c>
       <c r="D12" t="s">
         <v>18</v>
@@ -4109,7 +4216,7 @@
         <v>3</v>
       </c>
       <c r="K12" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L12" s="4">
         <v>2500</v>
@@ -4124,14 +4231,13 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="7">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="B13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
       </c>
       <c r="D13" t="s">
         <v>18</v>
@@ -4155,7 +4261,7 @@
         <v>3</v>
       </c>
       <c r="K13" s="4">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="L13" s="4">
         <v>2500</v>
@@ -4169,66 +4275,26 @@
       </c>
     </row>
     <row r="14" spans="1:14">
-      <c r="A14" s="7">
-        <v>46228</v>
-      </c>
-      <c r="B14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D14" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="6">
-        <v>5</v>
-      </c>
-      <c r="G14" s="6">
-        <v>8</v>
-      </c>
-      <c r="H14" s="6">
-        <v>1</v>
-      </c>
-      <c r="I14" s="6">
-        <v>1</v>
-      </c>
-      <c r="J14" s="6">
-        <v>3</v>
-      </c>
-      <c r="K14" s="4">
-        <v>2</v>
-      </c>
-      <c r="L14" s="4">
-        <v>2500</v>
-      </c>
-      <c r="M14" t="s">
-        <v>46</v>
-      </c>
-      <c r="N14">
-        <f>WEEKNUM(tblSales[[#This Row],[Date]],2)</f>
-        <v>30</v>
-      </c>
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="C15" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
-  <conditionalFormatting sqref="C17">
+  <conditionalFormatting sqref="C15">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND($A2="",COUNTA($A2:$M2)&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B14" xr:uid="{9DD528E4-FED7-5A4D-9879-F613E122D88A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B13" xr:uid="{9DD528E4-FED7-5A4D-9879-F613E122D88A}">
       <formula1>SalesReps</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D14" xr:uid="{5476F50E-F9A4-B940-87EC-2556D58F6B3C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D13" xr:uid="{5476F50E-F9A4-B940-87EC-2556D58F6B3C}">
       <formula1>Products</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E14" xr:uid="{C77FD214-0C0B-A84C-85CB-D67896C0D069}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E13" xr:uid="{C77FD214-0C0B-A84C-85CB-D67896C0D069}">
       <formula1>SalesStatus</formula1>
     </dataValidation>
   </dataValidations>
@@ -4244,19 +4310,19 @@
           <x14:formula1>
             <xm:f>Settings!$A$2:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B1 B15:B1048576</xm:sqref>
+          <xm:sqref>B1 B14:B1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CE5B47F4-9175-5B48-AC3A-5F662E73BAB2}">
           <x14:formula1>
             <xm:f>Settings!$D$2:$D$7</xm:f>
           </x14:formula1>
-          <xm:sqref>E1 E15:E1048576</xm:sqref>
+          <xm:sqref>E1 E14:E1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{08D9A091-89D2-8141-A5F9-B1F20530F99F}">
           <x14:formula1>
             <xm:f>Settings!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>D1 D15:D1048576</xm:sqref>
+          <xm:sqref>D1 D14:D1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4267,11 +4333,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFD47183-1C90-8D4B-B2ED-8B123B836864}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4283,20 +4349,16 @@
         <v>43</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="G1" s="46" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="47" t="s">
-        <v>51</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="str" cm="1">
@@ -4309,7 +4371,7 @@
       </c>
       <c r="B2" s="10">
         <f>SUMIFS(tblSales[Revenue],tblSales[Sales Rep],$A2)</f>
-        <v>8</v>
+        <v>8000</v>
       </c>
       <c r="C2">
         <f>SUMIFS(tblSales[Sales],tblSales[Sales Rep],$A2)</f>
@@ -4323,13 +4385,7 @@
         <f>SUMIFS(tblSales[Opportunities],tblSales[Sales Rep],$A2)</f>
         <v>4</v>
       </c>
-      <c r="G2" s="48">
-        <v>29</v>
-      </c>
-      <c r="H2">
-        <f>SUMIFS(tblSales[Revenue],tblSales[Week],G2)</f>
-        <v>14</v>
-      </c>
+      <c r="G2" s="15"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="str">
@@ -4341,27 +4397,21 @@
 tblSales[Sales Rep],
 A3
 )</f>
-        <v>6</v>
+        <v>4000</v>
       </c>
       <c r="C3">
         <f>SUMIFS(tblSales[Sales],tblSales[Sales Rep],$A3)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3">
         <f>SUMIFS(tblSales[Meetings],tblSales[Sales Rep],$A3)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <f>SUMIFS(tblSales[Opportunities],tblSales[Sales Rep],$A3)</f>
-        <v>3</v>
-      </c>
-      <c r="G3" s="48">
-        <v>29</v>
-      </c>
-      <c r="H3">
-        <f>SUMIFS(tblSales[Revenue],tblSales[Week],G3)</f>
-        <v>14</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G3" s="15"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="str">
@@ -4373,7 +4423,7 @@
 tblSales[Sales Rep],
 A4
 )</f>
-        <v>6</v>
+        <v>6000</v>
       </c>
       <c r="C4">
         <f>SUMIFS(tblSales[Sales],tblSales[Sales Rep],$A4)</f>
@@ -4387,13 +4437,7 @@
         <f>SUMIFS(tblSales[Opportunities],tblSales[Sales Rep],$A4)</f>
         <v>3</v>
       </c>
-      <c r="G4" s="48">
-        <v>29</v>
-      </c>
-      <c r="H4">
-        <f>SUMIFS(tblSales[Revenue],tblSales[Week],G4)</f>
-        <v>14</v>
-      </c>
+      <c r="G4" s="15"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="str">
@@ -4405,7 +4449,7 @@
 tblSales[Sales Rep],
 A5
 )</f>
-        <v>6</v>
+        <v>6000</v>
       </c>
       <c r="C5">
         <f>SUMIFS(tblSales[Sales],tblSales[Sales Rep],$A5)</f>
@@ -4419,16 +4463,20 @@
         <f>SUMIFS(tblSales[Opportunities],tblSales[Sales Rep],$A5)</f>
         <v>3</v>
       </c>
-      <c r="G5" s="48">
-        <v>29</v>
-      </c>
-      <c r="H5">
-        <f>SUMIFS(tblSales[Revenue],tblSales[Week],G5)</f>
-        <v>14</v>
-      </c>
+      <c r="G5" s="15"/>
     </row>
     <row r="9" spans="1:8">
       <c r="B9" s="2"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="str">
+        <f>INDEX(Summary!$A$2:$A$5,MATCH(MAX(Summary!$B$2:$B$5),Summary!$B$2:$B$5,0))</f>
+        <v>Emma Smith</v>
+      </c>
+      <c r="B11" s="13">
+        <f>MAX(Summary!$B$2:$B$5)</f>
+        <v>8000</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -4439,9 +4487,36 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC9E3C38-541F-5D4D-BA26-8A8B7F122A28}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" cm="1">
+        <f t="array" ref="A2:A3">_xlfn._xlws.SORT(_xlfn.UNIQUE(tblSales[Week]))</f>
+        <v>29</v>
+      </c>
+      <c r="B2" cm="1">
+        <f t="array" ref="B2:B3">SUMIFS(tblSales[Revenue],tblSales[Week],_xlfn.ANCHORARRAY(A2))</f>
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>12000</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4610,6 +4685,12 @@
       <c r="E6">
         <v>5</v>
       </c>
+      <c r="G6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
       <c r="J6" t="s">
         <v>32</v>
       </c>

</xml_diff>